<commit_message>
Mise à jour de l'application
</commit_message>
<xml_diff>
--- a/data/2026-2027/DonneesGPSPropres.xlsx
+++ b/data/2026-2027/DonneesGPSPropres.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christophergallo/Desktop/Application perso/data/2026-2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B094524D-17FB-F244-BC68-5DD3024AE686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BCF94E7-881E-F54D-BD6E-E8C4924D1696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16360" xr2:uid="{D839DFFF-AA38-2145-9D48-3C82EEA1EE91}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1846" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1912" uniqueCount="404">
   <si>
     <t>Temps joué</t>
   </si>
@@ -1211,6 +1211,42 @@
   </si>
   <si>
     <t>01:23:38</t>
+  </si>
+  <si>
+    <t>00:58:33</t>
+  </si>
+  <si>
+    <t>00:32:09</t>
+  </si>
+  <si>
+    <t>00:59:27</t>
+  </si>
+  <si>
+    <t>00:59:52</t>
+  </si>
+  <si>
+    <t>01:19:21</t>
+  </si>
+  <si>
+    <t>01:43:36</t>
+  </si>
+  <si>
+    <t>01:42:15</t>
+  </si>
+  <si>
+    <t>01:20:02</t>
+  </si>
+  <si>
+    <t>01:41:44</t>
+  </si>
+  <si>
+    <t>01:41:36</t>
+  </si>
+  <si>
+    <t>01:42:08</t>
+  </si>
+  <si>
+    <t>N1 J3 VS Nîmes 05/09/2026</t>
   </si>
 </sst>
 </file>
@@ -1585,7 +1621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3AE8228-0F81-ED4B-A4A4-4C340123FE2A}">
-  <dimension ref="A1:V355"/>
+  <dimension ref="A1:V366"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
@@ -24834,6 +24870,754 @@
         <v>11</v>
       </c>
     </row>
+    <row r="356" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A356" t="s">
+        <v>21</v>
+      </c>
+      <c r="B356" s="1">
+        <v>46269</v>
+      </c>
+      <c r="C356" t="s">
+        <v>19</v>
+      </c>
+      <c r="D356" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="E356" t="s">
+        <v>88</v>
+      </c>
+      <c r="F356" t="s">
+        <v>23</v>
+      </c>
+      <c r="G356" t="s">
+        <v>392</v>
+      </c>
+      <c r="H356">
+        <v>3.67</v>
+      </c>
+      <c r="I356">
+        <v>0.15</v>
+      </c>
+      <c r="J356">
+        <v>3.51</v>
+      </c>
+      <c r="K356">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="L356">
+        <v>0.02</v>
+      </c>
+      <c r="M356">
+        <v>0</v>
+      </c>
+      <c r="N356">
+        <v>0</v>
+      </c>
+      <c r="O356">
+        <v>0</v>
+      </c>
+      <c r="P356">
+        <v>3.66</v>
+      </c>
+      <c r="Q356">
+        <v>23.76</v>
+      </c>
+      <c r="R356">
+        <v>4.0199999999999996</v>
+      </c>
+      <c r="S356">
+        <v>11</v>
+      </c>
+      <c r="T356">
+        <v>2</v>
+      </c>
+      <c r="U356">
+        <v>8</v>
+      </c>
+      <c r="V356">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="357" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A357" t="s">
+        <v>21</v>
+      </c>
+      <c r="B357" s="1">
+        <v>46269</v>
+      </c>
+      <c r="C357" t="s">
+        <v>19</v>
+      </c>
+      <c r="D357" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="E357" t="s">
+        <v>29</v>
+      </c>
+      <c r="F357" t="s">
+        <v>25</v>
+      </c>
+      <c r="G357" t="s">
+        <v>393</v>
+      </c>
+      <c r="H357">
+        <v>3.16</v>
+      </c>
+      <c r="I357">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="J357">
+        <v>2.6</v>
+      </c>
+      <c r="K357">
+        <v>0.37</v>
+      </c>
+      <c r="L357">
+        <v>0.15</v>
+      </c>
+      <c r="M357">
+        <v>0.04</v>
+      </c>
+      <c r="N357">
+        <v>0</v>
+      </c>
+      <c r="O357">
+        <v>4</v>
+      </c>
+      <c r="P357">
+        <v>5.88</v>
+      </c>
+      <c r="Q357">
+        <v>27.05</v>
+      </c>
+      <c r="R357">
+        <v>4.32</v>
+      </c>
+      <c r="S357">
+        <v>26</v>
+      </c>
+      <c r="T357">
+        <v>3</v>
+      </c>
+      <c r="U357">
+        <v>17</v>
+      </c>
+      <c r="V357">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="358" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A358" t="s">
+        <v>21</v>
+      </c>
+      <c r="B358" s="1">
+        <v>46269</v>
+      </c>
+      <c r="C358" t="s">
+        <v>19</v>
+      </c>
+      <c r="D358" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="E358" t="s">
+        <v>90</v>
+      </c>
+      <c r="F358" t="s">
+        <v>100</v>
+      </c>
+      <c r="G358" t="s">
+        <v>394</v>
+      </c>
+      <c r="H358">
+        <v>4.63</v>
+      </c>
+      <c r="I358">
+        <v>0.34</v>
+      </c>
+      <c r="J358">
+        <v>4.28</v>
+      </c>
+      <c r="K358">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="L358">
+        <v>0.06</v>
+      </c>
+      <c r="M358">
+        <v>0.01</v>
+      </c>
+      <c r="N358">
+        <v>0</v>
+      </c>
+      <c r="O358">
+        <v>2</v>
+      </c>
+      <c r="P358">
+        <v>4.26</v>
+      </c>
+      <c r="Q358">
+        <v>26.4</v>
+      </c>
+      <c r="R358">
+        <v>6.18</v>
+      </c>
+      <c r="S358">
+        <v>39</v>
+      </c>
+      <c r="T358">
+        <v>16</v>
+      </c>
+      <c r="U358">
+        <v>28</v>
+      </c>
+      <c r="V358">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="359" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A359" t="s">
+        <v>21</v>
+      </c>
+      <c r="B359" s="1">
+        <v>46269</v>
+      </c>
+      <c r="C359" t="s">
+        <v>19</v>
+      </c>
+      <c r="D359" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="E359" t="s">
+        <v>37</v>
+      </c>
+      <c r="F359" t="s">
+        <v>26</v>
+      </c>
+      <c r="G359" t="s">
+        <v>395</v>
+      </c>
+      <c r="H359">
+        <v>4.54</v>
+      </c>
+      <c r="I359">
+        <v>0.34</v>
+      </c>
+      <c r="J359">
+        <v>4.2</v>
+      </c>
+      <c r="K359">
+        <v>0.3</v>
+      </c>
+      <c r="L359">
+        <v>0.05</v>
+      </c>
+      <c r="M359">
+        <v>0</v>
+      </c>
+      <c r="N359">
+        <v>0</v>
+      </c>
+      <c r="O359">
+        <v>0</v>
+      </c>
+      <c r="P359">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="Q359">
+        <v>22.98</v>
+      </c>
+      <c r="R359">
+        <v>4.75</v>
+      </c>
+      <c r="S359">
+        <v>12</v>
+      </c>
+      <c r="T359">
+        <v>7</v>
+      </c>
+      <c r="U359">
+        <v>16</v>
+      </c>
+      <c r="V359">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="360" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A360" t="s">
+        <v>403</v>
+      </c>
+      <c r="B360" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C360" t="s">
+        <v>19</v>
+      </c>
+      <c r="D360" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="E360" t="s">
+        <v>97</v>
+      </c>
+      <c r="F360" t="s">
+        <v>26</v>
+      </c>
+      <c r="G360" t="s">
+        <v>396</v>
+      </c>
+      <c r="H360">
+        <v>8.9499999999999993</v>
+      </c>
+      <c r="I360">
+        <v>1.17</v>
+      </c>
+      <c r="J360">
+        <v>7.76</v>
+      </c>
+      <c r="K360">
+        <v>0.95</v>
+      </c>
+      <c r="L360">
+        <v>0.21</v>
+      </c>
+      <c r="M360">
+        <v>0.03</v>
+      </c>
+      <c r="N360">
+        <v>0</v>
+      </c>
+      <c r="O360">
+        <v>2</v>
+      </c>
+      <c r="P360">
+        <v>6.72</v>
+      </c>
+      <c r="Q360">
+        <v>29.35</v>
+      </c>
+      <c r="R360">
+        <v>4.92</v>
+      </c>
+      <c r="S360">
+        <v>23</v>
+      </c>
+      <c r="T360">
+        <v>3</v>
+      </c>
+      <c r="U360">
+        <v>43</v>
+      </c>
+      <c r="V360">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="361" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A361" t="s">
+        <v>403</v>
+      </c>
+      <c r="B361" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C361" t="s">
+        <v>19</v>
+      </c>
+      <c r="D361" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="E361" t="s">
+        <v>30</v>
+      </c>
+      <c r="F361" t="s">
+        <v>27</v>
+      </c>
+      <c r="G361" t="s">
+        <v>397</v>
+      </c>
+      <c r="H361">
+        <v>10.97</v>
+      </c>
+      <c r="I361">
+        <v>1.62</v>
+      </c>
+      <c r="J361">
+        <v>9.33</v>
+      </c>
+      <c r="K361">
+        <v>1.22</v>
+      </c>
+      <c r="L361">
+        <v>0.23</v>
+      </c>
+      <c r="M361">
+        <v>0.17</v>
+      </c>
+      <c r="N361">
+        <v>0.02</v>
+      </c>
+      <c r="O361">
+        <v>9</v>
+      </c>
+      <c r="P361">
+        <v>6.25</v>
+      </c>
+      <c r="Q361">
+        <v>31.1</v>
+      </c>
+      <c r="R361">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="S361">
+        <v>34</v>
+      </c>
+      <c r="T361">
+        <v>7</v>
+      </c>
+      <c r="U361">
+        <v>36</v>
+      </c>
+      <c r="V361">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="362" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A362" t="s">
+        <v>403</v>
+      </c>
+      <c r="B362" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C362" t="s">
+        <v>19</v>
+      </c>
+      <c r="D362" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="E362" t="s">
+        <v>162</v>
+      </c>
+      <c r="F362" t="s">
+        <v>27</v>
+      </c>
+      <c r="G362" t="s">
+        <v>398</v>
+      </c>
+      <c r="H362">
+        <v>9.35</v>
+      </c>
+      <c r="I362">
+        <v>1.32</v>
+      </c>
+      <c r="J362">
+        <v>8.01</v>
+      </c>
+      <c r="K362">
+        <v>0.79</v>
+      </c>
+      <c r="L362">
+        <v>0.4</v>
+      </c>
+      <c r="M362">
+        <v>0.11</v>
+      </c>
+      <c r="N362">
+        <v>0.03</v>
+      </c>
+      <c r="O362">
+        <v>11</v>
+      </c>
+      <c r="P362">
+        <v>5.58</v>
+      </c>
+      <c r="Q362">
+        <v>33.409999999999997</v>
+      </c>
+      <c r="R362">
+        <v>4.17</v>
+      </c>
+      <c r="S362">
+        <v>35</v>
+      </c>
+      <c r="T362">
+        <v>3</v>
+      </c>
+      <c r="U362">
+        <v>33</v>
+      </c>
+      <c r="V362">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="363" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A363" t="s">
+        <v>403</v>
+      </c>
+      <c r="B363" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C363" t="s">
+        <v>19</v>
+      </c>
+      <c r="D363" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="E363" t="s">
+        <v>165</v>
+      </c>
+      <c r="F363" t="s">
+        <v>100</v>
+      </c>
+      <c r="G363" t="s">
+        <v>399</v>
+      </c>
+      <c r="H363">
+        <v>8.59</v>
+      </c>
+      <c r="I363">
+        <v>1.68</v>
+      </c>
+      <c r="J363">
+        <v>6.89</v>
+      </c>
+      <c r="K363">
+        <v>1.07</v>
+      </c>
+      <c r="L363">
+        <v>0.5</v>
+      </c>
+      <c r="M363">
+        <v>0.12</v>
+      </c>
+      <c r="N363">
+        <v>0.01</v>
+      </c>
+      <c r="O363">
+        <v>10</v>
+      </c>
+      <c r="P363">
+        <v>6.36</v>
+      </c>
+      <c r="Q363">
+        <v>31.53</v>
+      </c>
+      <c r="R363">
+        <v>4.92</v>
+      </c>
+      <c r="S363">
+        <v>49</v>
+      </c>
+      <c r="T363">
+        <v>8</v>
+      </c>
+      <c r="U363">
+        <v>32</v>
+      </c>
+      <c r="V363">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="364" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A364" t="s">
+        <v>403</v>
+      </c>
+      <c r="B364" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C364" t="s">
+        <v>19</v>
+      </c>
+      <c r="D364" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="E364" t="s">
+        <v>183</v>
+      </c>
+      <c r="F364" t="s">
+        <v>23</v>
+      </c>
+      <c r="G364" t="s">
+        <v>400</v>
+      </c>
+      <c r="H364">
+        <v>10.16</v>
+      </c>
+      <c r="I364">
+        <v>1.21</v>
+      </c>
+      <c r="J364">
+        <v>8.93</v>
+      </c>
+      <c r="K364">
+        <v>1</v>
+      </c>
+      <c r="L364">
+        <v>0.18</v>
+      </c>
+      <c r="M364">
+        <v>0.05</v>
+      </c>
+      <c r="N364">
+        <v>0</v>
+      </c>
+      <c r="O364">
+        <v>5</v>
+      </c>
+      <c r="P364">
+        <v>5.88</v>
+      </c>
+      <c r="Q364">
+        <v>28.97</v>
+      </c>
+      <c r="R364">
+        <v>5.28</v>
+      </c>
+      <c r="S364">
+        <v>47</v>
+      </c>
+      <c r="T364">
+        <v>7</v>
+      </c>
+      <c r="U364">
+        <v>29</v>
+      </c>
+      <c r="V364">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="365" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A365" t="s">
+        <v>403</v>
+      </c>
+      <c r="B365" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C365" t="s">
+        <v>19</v>
+      </c>
+      <c r="D365" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="E365" t="s">
+        <v>93</v>
+      </c>
+      <c r="F365" t="s">
+        <v>102</v>
+      </c>
+      <c r="G365" t="s">
+        <v>401</v>
+      </c>
+      <c r="H365">
+        <v>10.53</v>
+      </c>
+      <c r="I365">
+        <v>1.6</v>
+      </c>
+      <c r="J365">
+        <v>8.91</v>
+      </c>
+      <c r="K365">
+        <v>1.17</v>
+      </c>
+      <c r="L365">
+        <v>0.37</v>
+      </c>
+      <c r="M365">
+        <v>0.08</v>
+      </c>
+      <c r="N365">
+        <v>0</v>
+      </c>
+      <c r="O365">
+        <v>7</v>
+      </c>
+      <c r="P365">
+        <v>6.16</v>
+      </c>
+      <c r="Q365">
+        <v>29.64</v>
+      </c>
+      <c r="R365">
+        <v>4.76</v>
+      </c>
+      <c r="S365">
+        <v>48</v>
+      </c>
+      <c r="T365">
+        <v>5</v>
+      </c>
+      <c r="U365">
+        <v>39</v>
+      </c>
+      <c r="V365">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="366" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A366" t="s">
+        <v>403</v>
+      </c>
+      <c r="B366" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C366" t="s">
+        <v>19</v>
+      </c>
+      <c r="D366" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="E366" t="s">
+        <v>86</v>
+      </c>
+      <c r="F366" t="s">
+        <v>26</v>
+      </c>
+      <c r="G366" t="s">
+        <v>402</v>
+      </c>
+      <c r="H366">
+        <v>11.95</v>
+      </c>
+      <c r="I366">
+        <v>2.36</v>
+      </c>
+      <c r="J366">
+        <v>9.56</v>
+      </c>
+      <c r="K366">
+        <v>1.72</v>
+      </c>
+      <c r="L366">
+        <v>0.61</v>
+      </c>
+      <c r="M366">
+        <v>0.05</v>
+      </c>
+      <c r="N366">
+        <v>0</v>
+      </c>
+      <c r="O366">
+        <v>7</v>
+      </c>
+      <c r="P366">
+        <v>7.01</v>
+      </c>
+      <c r="Q366">
+        <v>26.98</v>
+      </c>
+      <c r="R366">
+        <v>4.8099999999999996</v>
+      </c>
+      <c r="S366">
+        <v>48</v>
+      </c>
+      <c r="T366">
+        <v>9</v>
+      </c>
+      <c r="U366">
+        <v>44</v>
+      </c>
+      <c r="V366">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>